<commit_message>
Se modifica código para integrar a incio y final de matriz puntos equivalentes a "Inóculo" y "Descube" en función de muestras declaradas como tal en SW (columna muestreo_text).
</commit_message>
<xml_diff>
--- a/Datos Experimentales/Data 24021.xlsx
+++ b/Datos Experimentales/Data 24021.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cltor\Documents\SB_Calibration_2025\Datos Experimentales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04E49C16-F97D-4833-9963-2C9D76C1B548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{827A841F-6997-4468-9CC5-4C4E187F0090}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="998" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="998" uniqueCount="325">
   <si>
     <t>parametro</t>
   </si>
@@ -1005,14 +1005,25 @@
   </si>
   <si>
     <t>volumen</t>
+  </si>
+  <si>
+    <t>4. Descube</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1040,9 +1051,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1383,9 +1395,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B106"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1393,7 +1405,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1401,7 +1413,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1409,7 +1421,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1417,7 +1429,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -1425,7 +1437,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1433,7 +1445,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1441,7 +1453,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -1449,7 +1461,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -1457,7 +1469,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -1465,7 +1477,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -1473,7 +1485,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -1481,7 +1493,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -1489,7 +1501,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -1497,7 +1509,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -1505,7 +1517,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>18</v>
       </c>
@@ -1513,7 +1525,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>19</v>
       </c>
@@ -1521,7 +1533,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -1529,7 +1541,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -1537,7 +1549,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>22</v>
       </c>
@@ -1545,7 +1557,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>23</v>
       </c>
@@ -1553,7 +1565,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>24</v>
       </c>
@@ -1561,7 +1573,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>25</v>
       </c>
@@ -1569,7 +1581,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>26</v>
       </c>
@@ -1577,7 +1589,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>27</v>
       </c>
@@ -1585,7 +1597,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>28</v>
       </c>
@@ -1593,7 +1605,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>29</v>
       </c>
@@ -1601,7 +1613,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>30</v>
       </c>
@@ -1609,7 +1621,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>31</v>
       </c>
@@ -1617,7 +1629,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>33</v>
       </c>
@@ -1625,7 +1637,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>34</v>
       </c>
@@ -1633,7 +1645,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>35</v>
       </c>
@@ -1641,7 +1653,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>36</v>
       </c>
@@ -1649,7 +1661,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>37</v>
       </c>
@@ -1657,7 +1669,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>39</v>
       </c>
@@ -1665,7 +1677,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>40</v>
       </c>
@@ -1673,7 +1685,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -1681,7 +1693,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -1689,7 +1701,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -1697,7 +1709,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -1705,7 +1717,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -1713,7 +1725,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>46</v>
       </c>
@@ -1721,7 +1733,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>47</v>
       </c>
@@ -1729,7 +1741,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>49</v>
       </c>
@@ -1737,7 +1749,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>50</v>
       </c>
@@ -1745,7 +1757,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>51</v>
       </c>
@@ -1753,7 +1765,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>52</v>
       </c>
@@ -1761,7 +1773,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>54</v>
       </c>
@@ -1769,7 +1781,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>55</v>
       </c>
@@ -1777,7 +1789,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>56</v>
       </c>
@@ -1785,7 +1797,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>57</v>
       </c>
@@ -1793,7 +1805,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>58</v>
       </c>
@@ -1801,7 +1813,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>59</v>
       </c>
@@ -1809,7 +1821,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>61</v>
       </c>
@@ -1817,7 +1829,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>62</v>
       </c>
@@ -1825,7 +1837,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>63</v>
       </c>
@@ -1833,7 +1845,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>64</v>
       </c>
@@ -1841,7 +1853,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>65</v>
       </c>
@@ -1849,7 +1861,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>67</v>
       </c>
@@ -1857,7 +1869,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>68</v>
       </c>
@@ -1865,7 +1877,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="61" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>69</v>
       </c>
@@ -1873,7 +1885,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="62" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>70</v>
       </c>
@@ -1881,7 +1893,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="63" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>71</v>
       </c>
@@ -1889,7 +1901,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="64" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>72</v>
       </c>
@@ -1897,7 +1909,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="65" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>73</v>
       </c>
@@ -1905,7 +1917,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="66" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>74</v>
       </c>
@@ -1913,7 +1925,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="67" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>75</v>
       </c>
@@ -1921,7 +1933,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="68" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>77</v>
       </c>
@@ -1929,7 +1941,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="69" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>79</v>
       </c>
@@ -1937,7 +1949,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="70" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>80</v>
       </c>
@@ -1945,7 +1957,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="71" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>81</v>
       </c>
@@ -1953,7 +1965,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="72" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>83</v>
       </c>
@@ -1961,7 +1973,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="73" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>84</v>
       </c>
@@ -1969,7 +1981,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="74" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>85</v>
       </c>
@@ -1977,7 +1989,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="75" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>86</v>
       </c>
@@ -1985,7 +1997,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="76" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>87</v>
       </c>
@@ -1993,7 +2005,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="77" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>88</v>
       </c>
@@ -2001,7 +2013,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="78" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>89</v>
       </c>
@@ -2009,7 +2021,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="79" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>90</v>
       </c>
@@ -2017,7 +2029,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="80" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>91</v>
       </c>
@@ -2025,7 +2037,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="81" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>92</v>
       </c>
@@ -2033,7 +2045,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="82" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>93</v>
       </c>
@@ -2041,7 +2053,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="83" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>94</v>
       </c>
@@ -2049,7 +2061,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="84" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>95</v>
       </c>
@@ -2057,7 +2069,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="85" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>96</v>
       </c>
@@ -2065,7 +2077,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="86" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>97</v>
       </c>
@@ -2073,7 +2085,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="87" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>99</v>
       </c>
@@ -2081,7 +2093,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="88" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>100</v>
       </c>
@@ -2089,7 +2101,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="89" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>101</v>
       </c>
@@ -2097,7 +2109,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="90" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>102</v>
       </c>
@@ -2105,7 +2117,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="91" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>103</v>
       </c>
@@ -2113,7 +2125,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="92" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>104</v>
       </c>
@@ -2121,7 +2133,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="93" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>105</v>
       </c>
@@ -2129,7 +2141,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="94" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>106</v>
       </c>
@@ -2137,7 +2149,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="95" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>107</v>
       </c>
@@ -2145,7 +2157,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="96" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>108</v>
       </c>
@@ -2153,7 +2165,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="97" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>109</v>
       </c>
@@ -2161,7 +2173,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="98" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>110</v>
       </c>
@@ -2169,7 +2181,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="99" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>111</v>
       </c>
@@ -2177,7 +2189,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="100" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>112</v>
       </c>
@@ -2185,7 +2197,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="101" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>113</v>
       </c>
@@ -2193,7 +2205,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="102" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>115</v>
       </c>
@@ -2201,7 +2213,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="103" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>116</v>
       </c>
@@ -2209,7 +2221,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="104" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>117</v>
       </c>
@@ -2217,7 +2229,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="105" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>118</v>
       </c>
@@ -2225,7 +2237,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="106" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>119</v>
       </c>
@@ -2244,7 +2256,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -2256,9 +2268,9 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>269</v>
       </c>
@@ -2289,9 +2301,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:C45"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>274</v>
       </c>
@@ -2302,7 +2314,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>277</v>
       </c>
@@ -2313,7 +2325,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>278</v>
       </c>
@@ -2324,7 +2336,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>279</v>
       </c>
@@ -2335,7 +2347,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>280</v>
       </c>
@@ -2346,7 +2358,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>281</v>
       </c>
@@ -2357,7 +2369,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>282</v>
       </c>
@@ -2368,7 +2380,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>283</v>
       </c>
@@ -2379,7 +2391,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>284</v>
       </c>
@@ -2390,7 +2402,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>285</v>
       </c>
@@ -2401,7 +2413,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>286</v>
       </c>
@@ -2412,7 +2424,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>287</v>
       </c>
@@ -2423,7 +2435,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>288</v>
       </c>
@@ -2434,7 +2446,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>289</v>
       </c>
@@ -2445,7 +2457,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>290</v>
       </c>
@@ -2456,7 +2468,7 @@
         <v>16.2</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>291</v>
       </c>
@@ -2467,7 +2479,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>292</v>
       </c>
@@ -2478,7 +2490,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>293</v>
       </c>
@@ -2489,7 +2501,7 @@
         <v>16.7</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>294</v>
       </c>
@@ -2500,7 +2512,7 @@
         <v>16.600000000000001</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>295</v>
       </c>
@@ -2511,7 +2523,7 @@
         <v>16.600000000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>296</v>
       </c>
@@ -2522,7 +2534,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>297</v>
       </c>
@@ -2533,7 +2545,7 @@
         <v>16.8</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>298</v>
       </c>
@@ -2544,7 +2556,7 @@
         <v>16.600000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>299</v>
       </c>
@@ -2555,7 +2567,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>300</v>
       </c>
@@ -2566,7 +2578,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>301</v>
       </c>
@@ -2577,7 +2589,7 @@
         <v>16.600000000000001</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>302</v>
       </c>
@@ -2588,7 +2600,7 @@
         <v>16.600000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>303</v>
       </c>
@@ -2599,7 +2611,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>304</v>
       </c>
@@ -2610,7 +2622,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>305</v>
       </c>
@@ -2621,7 +2633,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>306</v>
       </c>
@@ -2632,7 +2644,7 @@
         <v>16.8</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>307</v>
       </c>
@@ -2643,7 +2655,7 @@
         <v>17.5</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>308</v>
       </c>
@@ -2654,7 +2666,7 @@
         <v>17.399999999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>309</v>
       </c>
@@ -2665,7 +2677,7 @@
         <v>16.2</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>310</v>
       </c>
@@ -2676,7 +2688,7 @@
         <v>17.2</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>311</v>
       </c>
@@ -2687,7 +2699,7 @@
         <v>16.7</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>312</v>
       </c>
@@ -2698,7 +2710,7 @@
         <v>16.3</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>313</v>
       </c>
@@ -2709,7 +2721,7 @@
         <v>17.399999999999999</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>314</v>
       </c>
@@ -2720,7 +2732,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>315</v>
       </c>
@@ -2731,7 +2743,7 @@
         <v>16.7</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>316</v>
       </c>
@@ -2742,7 +2754,7 @@
         <v>17.2</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>317</v>
       </c>
@@ -2753,7 +2765,7 @@
         <v>16.3</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>318</v>
       </c>
@@ -2764,7 +2776,7 @@
         <v>16.899999999999999</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>319</v>
       </c>
@@ -2775,7 +2787,7 @@
         <v>17.399999999999999</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>320</v>
       </c>
@@ -2797,9 +2809,9 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:C45"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>274</v>
       </c>
@@ -2810,7 +2822,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>277</v>
       </c>
@@ -2821,7 +2833,7 @@
         <v>1086</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>278</v>
       </c>
@@ -2832,7 +2844,7 @@
         <v>1086</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>279</v>
       </c>
@@ -2843,7 +2855,7 @@
         <v>1086</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>280</v>
       </c>
@@ -2854,7 +2866,7 @@
         <v>1083</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>281</v>
       </c>
@@ -2865,7 +2877,7 @@
         <v>1083</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>282</v>
       </c>
@@ -2876,7 +2888,7 @@
         <v>1077</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>283</v>
       </c>
@@ -2887,7 +2899,7 @@
         <v>1073</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>284</v>
       </c>
@@ -2898,7 +2910,7 @@
         <v>1067</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>285</v>
       </c>
@@ -2909,7 +2921,7 @@
         <v>1062</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>286</v>
       </c>
@@ -2920,7 +2932,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>287</v>
       </c>
@@ -2931,7 +2943,7 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>288</v>
       </c>
@@ -2942,7 +2954,7 @@
         <v>1043</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>289</v>
       </c>
@@ -2953,7 +2965,7 @@
         <v>1040</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>290</v>
       </c>
@@ -2964,7 +2976,7 @@
         <v>1035</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>291</v>
       </c>
@@ -2975,7 +2987,7 @@
         <v>1030</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>292</v>
       </c>
@@ -2986,7 +2998,7 @@
         <v>1029</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>293</v>
       </c>
@@ -2997,7 +3009,7 @@
         <v>1027</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>294</v>
       </c>
@@ -3008,7 +3020,7 @@
         <v>1021</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>295</v>
       </c>
@@ -3019,7 +3031,7 @@
         <v>1018</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>296</v>
       </c>
@@ -3030,7 +3042,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>297</v>
       </c>
@@ -3041,7 +3053,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>298</v>
       </c>
@@ -3052,7 +3064,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>299</v>
       </c>
@@ -3063,7 +3075,7 @@
         <v>1009</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>300</v>
       </c>
@@ -3074,7 +3086,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>301</v>
       </c>
@@ -3085,7 +3097,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>302</v>
       </c>
@@ -3096,7 +3108,7 @@
         <v>1005</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>303</v>
       </c>
@@ -3107,7 +3119,7 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>304</v>
       </c>
@@ -3118,7 +3130,7 @@
         <v>1003</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>305</v>
       </c>
@@ -3129,7 +3141,7 @@
         <v>1002</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>306</v>
       </c>
@@ -3140,7 +3152,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>307</v>
       </c>
@@ -3151,7 +3163,7 @@
         <v>999</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>308</v>
       </c>
@@ -3162,7 +3174,7 @@
         <v>999</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>309</v>
       </c>
@@ -3173,7 +3185,7 @@
         <v>999</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>310</v>
       </c>
@@ -3184,7 +3196,7 @@
         <v>997</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>311</v>
       </c>
@@ -3195,7 +3207,7 @@
         <v>997</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>312</v>
       </c>
@@ -3206,7 +3218,7 @@
         <v>996</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>313</v>
       </c>
@@ -3217,7 +3229,7 @@
         <v>995</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>314</v>
       </c>
@@ -3228,7 +3240,7 @@
         <v>995</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>315</v>
       </c>
@@ -3239,7 +3251,7 @@
         <v>995</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>316</v>
       </c>
@@ -3250,7 +3262,7 @@
         <v>995</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>317</v>
       </c>
@@ -3261,7 +3273,7 @@
         <v>993</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>318</v>
       </c>
@@ -3272,7 +3284,7 @@
         <v>993</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>319</v>
       </c>
@@ -3283,7 +3295,7 @@
         <v>993</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>320</v>
       </c>
@@ -3305,9 +3317,9 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>274</v>
       </c>
@@ -3341,9 +3353,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:CO2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:93" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:93" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -3624,7 +3636,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="2" spans="1:93" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:93" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>9841</v>
       </c>
@@ -3895,9 +3907,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Q12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>142</v>
       </c>
@@ -3950,7 +3962,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>9841</v>
       </c>
@@ -3979,7 +3991,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>9841</v>
       </c>
@@ -4014,7 +4026,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>9841</v>
       </c>
@@ -4043,7 +4055,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>9841</v>
       </c>
@@ -4093,7 +4105,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>9841</v>
       </c>
@@ -4143,7 +4155,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>9841</v>
       </c>
@@ -4178,7 +4190,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>9841</v>
       </c>
@@ -4225,7 +4237,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>9841</v>
       </c>
@@ -4254,7 +4266,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9841</v>
       </c>
@@ -4289,7 +4301,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9841</v>
       </c>
@@ -4324,7 +4336,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>9841</v>
       </c>
@@ -4370,9 +4382,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>142</v>
       </c>
@@ -4404,7 +4416,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>9841</v>
       </c>
@@ -4436,7 +4448,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>9841</v>
       </c>
@@ -4468,7 +4480,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>9841</v>
       </c>
@@ -4511,7 +4523,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -4523,9 +4535,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:J2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>142</v>
       </c>
@@ -4557,7 +4569,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>9841</v>
       </c>
@@ -4600,9 +4612,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>142</v>
       </c>
@@ -4619,7 +4631,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>9841</v>
       </c>
@@ -4641,7 +4653,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -4653,9 +4665,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:P36"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>142</v>
       </c>
@@ -4705,7 +4717,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>9841</v>
       </c>
@@ -4755,7 +4767,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>9841</v>
       </c>
@@ -4805,7 +4817,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>9841</v>
       </c>
@@ -4855,7 +4867,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>9841</v>
       </c>
@@ -4905,7 +4917,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>9841</v>
       </c>
@@ -4955,7 +4967,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>9841</v>
       </c>
@@ -5005,7 +5017,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>9841</v>
       </c>
@@ -5055,7 +5067,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>9841</v>
       </c>
@@ -5105,7 +5117,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9841</v>
       </c>
@@ -5155,7 +5167,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9841</v>
       </c>
@@ -5205,7 +5217,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>9841</v>
       </c>
@@ -5255,7 +5267,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>9841</v>
       </c>
@@ -5305,7 +5317,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>9841</v>
       </c>
@@ -5355,7 +5367,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>9841</v>
       </c>
@@ -5405,7 +5417,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>9841</v>
       </c>
@@ -5455,7 +5467,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>9841</v>
       </c>
@@ -5505,7 +5517,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>9841</v>
       </c>
@@ -5555,7 +5567,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>9841</v>
       </c>
@@ -5574,7 +5586,7 @@
       <c r="F19" t="s">
         <v>123</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G19" s="2" t="s">
         <v>120</v>
       </c>
       <c r="H19" t="s">
@@ -5605,7 +5617,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>9841</v>
       </c>
@@ -5655,7 +5667,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>9841</v>
       </c>
@@ -5705,7 +5717,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>9841</v>
       </c>
@@ -5755,7 +5767,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>9841</v>
       </c>
@@ -5805,7 +5817,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>9841</v>
       </c>
@@ -5855,7 +5867,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>9841</v>
       </c>
@@ -5905,7 +5917,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>9841</v>
       </c>
@@ -5955,7 +5967,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>9841</v>
       </c>
@@ -5984,7 +5996,7 @@
         <v>233</v>
       </c>
       <c r="J27" t="s">
-        <v>234</v>
+        <v>324</v>
       </c>
       <c r="K27" t="s">
         <v>235</v>
@@ -6005,7 +6017,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="28" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>9841</v>
       </c>
@@ -6034,7 +6046,7 @@
         <v>233</v>
       </c>
       <c r="J28" t="s">
-        <v>234</v>
+        <v>324</v>
       </c>
       <c r="K28" t="s">
         <v>248</v>
@@ -6055,7 +6067,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="29" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>9841</v>
       </c>
@@ -6084,7 +6096,7 @@
         <v>233</v>
       </c>
       <c r="J29" t="s">
-        <v>234</v>
+        <v>324</v>
       </c>
       <c r="K29" t="s">
         <v>250</v>
@@ -6105,7 +6117,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>9841</v>
       </c>
@@ -6134,7 +6146,7 @@
         <v>233</v>
       </c>
       <c r="J30" t="s">
-        <v>234</v>
+        <v>324</v>
       </c>
       <c r="K30" t="s">
         <v>244</v>
@@ -6155,7 +6167,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>9841</v>
       </c>
@@ -6184,7 +6196,7 @@
         <v>233</v>
       </c>
       <c r="J31" t="s">
-        <v>234</v>
+        <v>324</v>
       </c>
       <c r="K31" t="s">
         <v>264</v>
@@ -6205,7 +6217,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>9841</v>
       </c>
@@ -6234,7 +6246,7 @@
         <v>233</v>
       </c>
       <c r="J32" t="s">
-        <v>234</v>
+        <v>324</v>
       </c>
       <c r="K32" t="s">
         <v>253</v>
@@ -6255,7 +6267,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="33" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>9841</v>
       </c>
@@ -6284,7 +6296,7 @@
         <v>233</v>
       </c>
       <c r="J33" t="s">
-        <v>234</v>
+        <v>324</v>
       </c>
       <c r="K33" t="s">
         <v>255</v>
@@ -6305,7 +6317,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="34" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>9841</v>
       </c>
@@ -6334,7 +6346,7 @@
         <v>233</v>
       </c>
       <c r="J34" t="s">
-        <v>234</v>
+        <v>324</v>
       </c>
       <c r="K34" t="s">
         <v>229</v>
@@ -6355,7 +6367,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="35" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>9841</v>
       </c>
@@ -6384,7 +6396,7 @@
         <v>233</v>
       </c>
       <c r="J35" t="s">
-        <v>234</v>
+        <v>324</v>
       </c>
       <c r="K35" t="s">
         <v>240</v>
@@ -6405,7 +6417,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="36" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>9841</v>
       </c>
@@ -6434,7 +6446,7 @@
         <v>233</v>
       </c>
       <c r="J36" t="s">
-        <v>234</v>
+        <v>324</v>
       </c>
       <c r="K36" t="s">
         <v>241</v>
@@ -6458,7 +6470,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:P8 A16:P36 A9:D9 F9:P9 A10:D15 F10:P15" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:P8 A16:P26 A9:D9 F9:P9 A10:D15 F10:P15 A27:I36 K27:P36" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>